<commit_message>
fix: adcode lookup prefers city-level codes over districts (澳門 820000)
</commit_message>
<xml_diff>
--- a/AMap_adcode_citycode.xlsx
+++ b/AMap_adcode_citycode.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liusilin/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\nicklam-ai\repos\wepush-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E445125-55F7-B545-B14B-F44E0515580B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BAC1DF7-BFD9-44C3-8861-35D5AA6DEC53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6120" yWindow="6420" windowWidth="22820" windowHeight="14260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -30,6 +30,9 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -20500,7 +20503,7 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="宋体"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -20511,7 +20514,7 @@
     </font>
     <font>
       <sz val="9"/>
-      <name val="宋体"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -20519,7 +20522,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -20527,7 +20530,7 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="宋体"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -20571,18 +20574,10 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Santa" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -20914,9 +20909,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E3241"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="4" width="17.1640625" customWidth="1"/>
+    <col min="1" max="4" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15" customHeight="1">
@@ -56579,14 +56574,14 @@
     <sortCondition ref="B2:B3281"/>
   </sortState>
   <phoneticPr fontId="2" type="noConversion"/>
+  <conditionalFormatting sqref="B1">
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B2">
-    <cfRule type="duplicateValues" dxfId="3" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B3242 B3288:B1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B1">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>